<commit_message>
📊 Auto update: 2026-06-01
</commit_message>
<xml_diff>
--- a/docs/data.xlsx
+++ b/docs/data.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>업데이트: 2026-05-06 | Yahoo Finance Price Return</t>
+          <t>업데이트: 2026-06-01 | Yahoo Finance Price Return</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>2026</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>6.04</v>
+        <v>10.73</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>10.95</v>
+        <v>20.13</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>64.61</v>
+        <v>101.13</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>3.75</v>
@@ -1150,13 +1150,13 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>9.006</v>
+        <v>9.237</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>14.895</v>
+        <v>15.344</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>8.233000000000001</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="31">
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.836</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>1.304</v>
+        <v>1.339</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.842</v>
+        <v>0.9379999999999999</v>
       </c>
     </row>
     <row r="32">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>15.151</v>
+        <v>15.182</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>18.377</v>
+        <v>18.489</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>21.025</v>
+        <v>21.875</v>
       </c>
     </row>
     <row r="33">
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>0.648</v>
+        <v>0.661</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.852</v>
+        <v>0.869</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.481</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="34">
@@ -5215,13 +5215,13 @@
         </is>
       </c>
       <c r="B248" s="14" t="n">
-        <v>0.7</v>
+        <v>5.15</v>
       </c>
       <c r="C248" s="14" t="n">
-        <v>2.05</v>
+        <v>10.49</v>
       </c>
       <c r="D248" s="14" t="n">
-        <v>5.12</v>
+        <v>28.45</v>
       </c>
     </row>
   </sheetData>
@@ -5299,13 +5299,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.8175565119617104</v>
+        <v>0.835721980246931</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1.304455368577213</v>
+        <v>1.338921599506757</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.8423404870400044</v>
+        <v>0.9375429420129839</v>
       </c>
     </row>
     <row r="6">
@@ -5315,7 +5315,7 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>1.312815216695795</v>
+        <v>1.366295890092029</v>
       </c>
       <c r="C6" s="18" t="n">
         <v>1.850183334037547</v>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4.373817203234671</v>
+        <v>4.382545697474485</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>5.304979080771218</v>
+        <v>5.33717998298398</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>6.069376734460171</v>
+        <v>6.314781555736555</v>
       </c>
     </row>
     <row r="8">
@@ -5347,13 +5347,13 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>15.15134723804252</v>
+        <v>15.18158362903638</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>18.37698660197157</v>
+        <v>18.4885337993357</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>21.02493774872299</v>
+        <v>21.8750449864691</v>
       </c>
     </row>
     <row r="9">
@@ -5439,13 +5439,13 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-0.5768004906746571</v>
+        <v>-0.5819144009370661</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-0.3560521299514313</v>
+        <v>-0.3480928704733733</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.4298456868179507</v>
+        <v>0.6799959054361719</v>
       </c>
     </row>
     <row r="14">
@@ -5455,13 +5455,13 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.202639035368419</v>
+        <v>1.182664866928891</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>0.5602678414379256</v>
+        <v>0.5200429945751837</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>4.276803686916082</v>
+        <v>4.694653627306373</v>
       </c>
     </row>
     <row r="15">
@@ -5519,13 +5519,13 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>9.005533622973116</v>
+        <v>9.236685227718834</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>14.8953215793612</v>
+        <v>15.34358155558952</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>8.232753925626724</v>
+        <v>9.300282356563683</v>
       </c>
     </row>
     <row r="19">
@@ -5535,13 +5535,13 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>0.6475119333881768</v>
+        <v>0.6605808727214922</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>0.851797128765778</v>
+        <v>0.8690283052438901</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.4807665052465612</v>
+        <v>0.5143082133597832</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Auto update: 2026-07-01
</commit_message>
<xml_diff>
--- a/docs/data.xlsx
+++ b/docs/data.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>업데이트: 2026-06-01 | Yahoo Finance Price Return</t>
+          <t>업데이트: 2026-07-01 | Yahoo Finance Price Return</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>2026</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>10.73</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>20.13</v>
+        <v>19.91</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>101.13</v>
+        <v>99.2</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>3.75</v>
@@ -1150,13 +1150,13 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>9.237</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>15.344</v>
+        <v>15.266</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>9.300000000000001</v>
+        <v>9.209</v>
       </c>
     </row>
     <row r="31">
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.836</v>
+        <v>0.828</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>1.339</v>
+        <v>1.333</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="32">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>15.182</v>
+        <v>15.156</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>18.489</v>
+        <v>18.454</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>21.875</v>
+        <v>21.834</v>
       </c>
     </row>
     <row r="33">
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>0.661</v>
+        <v>0.656</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.869</v>
+        <v>0.867</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.514</v>
+        <v>0.511</v>
       </c>
     </row>
     <row r="34">
@@ -1266,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D248"/>
+  <dimension ref="A1:D249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>월간 수익률 (2006.1 ~ 2026.05)</t>
+          <t>월간 수익률 (2006.1 ~ 2026.06)</t>
         </is>
       </c>
     </row>
@@ -5222,6 +5222,22 @@
       </c>
       <c r="D248" s="14" t="n">
         <v>28.45</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B249" s="15" t="n">
+        <v>-1.06</v>
+      </c>
+      <c r="C249" s="15" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="D249" s="15" t="n">
+        <v>-0.96</v>
       </c>
     </row>
   </sheetData>
@@ -5283,13 +5299,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5">
@@ -5299,13 +5315,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.835721980246931</v>
+        <v>0.8279969399178321</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1.338921599506757</v>
+        <v>1.332717205631521</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.9375429420129839</v>
+        <v>0.9298231682602658</v>
       </c>
     </row>
     <row r="6">
@@ -5315,13 +5331,13 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>1.366295890092029</v>
+        <v>1.339555553393912</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1.850183334037547</v>
+        <v>1.845703419189093</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.838264280160117</v>
+        <v>0.8352827572794652</v>
       </c>
     </row>
     <row r="7">
@@ -5331,13 +5347,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4.382545697474485</v>
+        <v>4.375270554592898</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>5.33717998298398</v>
+        <v>5.327165523218869</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>6.314781555736555</v>
+        <v>6.303044134196812</v>
       </c>
     </row>
     <row r="8">
@@ -5347,13 +5363,13 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>15.18158362903638</v>
+        <v>15.15638179482992</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>18.4885337993357</v>
+        <v>18.45384269308865</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>21.8750449864691</v>
+        <v>21.83438536555573</v>
       </c>
     </row>
     <row r="9">
@@ -5439,13 +5455,13 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-0.5819144009370661</v>
+        <v>-0.5774124374456441</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-0.3480928704733733</v>
+        <v>-0.3451933368953879</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.6799959054361719</v>
+        <v>0.6845798786689348</v>
       </c>
     </row>
     <row r="14">
@@ -5455,13 +5471,13 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.182664866928891</v>
+        <v>1.189176672035206</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>0.5200429945751837</v>
+        <v>0.5304190741117845</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>4.694653627306373</v>
+        <v>4.723422111329421</v>
       </c>
     </row>
     <row r="15">
@@ -5471,13 +5487,13 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>65.71428571428571</v>
+        <v>65.44715447154471</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>62.85714285714285</v>
+        <v>62.60162601626016</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>56.73469387755102</v>
+        <v>56.50406504065041</v>
       </c>
     </row>
     <row r="16">
@@ -5487,13 +5503,13 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>-7.423163148714707</v>
+        <v>-7.407727877425641</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>-8.256485496201039</v>
+        <v>-8.22106512846848</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>-7.672293658919779</v>
+        <v>-7.667102791213967</v>
       </c>
     </row>
     <row r="17">
@@ -5519,13 +5535,13 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>9.236685227718834</v>
+        <v>9.14046246715008</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>15.34358155558952</v>
+        <v>15.26612605843283</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>9.300282356563683</v>
+        <v>9.209294593663998</v>
       </c>
     </row>
     <row r="19">
@@ -5535,13 +5551,13 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>0.6605808727214922</v>
+        <v>0.6555630105862931</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>0.8690283052438901</v>
+        <v>0.8666274408835086</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.5143082133597832</v>
+        <v>0.511023224712568</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Auto update: 2026-08-01
</commit_message>
<xml_diff>
--- a/docs/data.xlsx
+++ b/docs/data.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>업데이트: 2026-07-01 | Yahoo Finance Price Return</t>
+          <t>업데이트: 2026-08-01 | Yahoo Finance Price Return</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>2026</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>9.550000000000001</v>
+        <v>9.41</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>19.91</v>
+        <v>11.98</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>99.2</v>
+        <v>32.73</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>3.75</v>
@@ -1150,13 +1150,13 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>9.140000000000001</v>
+        <v>9.095000000000001</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>15.266</v>
+        <v>14.818</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>9.209</v>
+        <v>7.038</v>
       </c>
     </row>
     <row r="31">
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.828</v>
+        <v>0.824</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>1.333</v>
+        <v>1.301</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.93</v>
+        <v>0.792</v>
       </c>
     </row>
     <row r="32">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>15.156</v>
+        <v>15.127</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>18.454</v>
+        <v>18.499</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>21.834</v>
+        <v>23.108</v>
       </c>
     </row>
     <row r="33">
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>0.656</v>
+        <v>0.654</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.867</v>
+        <v>0.844</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.511</v>
+        <v>0.411</v>
       </c>
     </row>
     <row r="34">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>2008-10 (-23.13%)</t>
+          <t>2026-07 (-34.01%)</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>월간 수익률 (2006.1 ~ 2026.06)</t>
+          <t>월간 수익률 (2006.1 ~ 2026.07)</t>
         </is>
       </c>
     </row>
@@ -5236,8 +5236,24 @@
       <c r="C249" s="15" t="n">
         <v>-0.19</v>
       </c>
-      <c r="D249" s="15" t="n">
-        <v>-0.96</v>
+      <c r="D249" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B250" s="15" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="C250" s="15" t="n">
+        <v>-6.61</v>
+      </c>
+      <c r="D250" s="15" t="n">
+        <v>-34.01</v>
       </c>
     </row>
   </sheetData>
@@ -5299,13 +5315,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5">
@@ -5315,13 +5331,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.8279969399178321</v>
+        <v>0.8241243222789321</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1.332717205631521</v>
+        <v>1.300548612970375</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.9298231682602658</v>
+        <v>0.792271644629278</v>
       </c>
     </row>
     <row r="6">
@@ -5331,13 +5347,13 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>1.339555553393912</v>
+        <v>1.312815216695795</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1.845703419189093</v>
+        <v>1.841223504340639</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.8352827572794652</v>
+        <v>0.8323012343988134</v>
       </c>
     </row>
     <row r="7">
@@ -5347,13 +5363,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4.375270554592898</v>
+        <v>4.366792837294682</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>5.327165523218869</v>
+        <v>5.340312017369913</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>6.303044134196812</v>
+        <v>6.670803021950943</v>
       </c>
     </row>
     <row r="8">
@@ -5363,13 +5379,13 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>15.15638179482992</v>
+        <v>15.12701412064448</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>18.45384269308865</v>
+        <v>18.49938348471067</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>21.83438536555573</v>
+        <v>23.10833952260607</v>
       </c>
     </row>
     <row r="9">
@@ -5385,7 +5401,7 @@
         <v>-16.2953145739305</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>-23.13439957216467</v>
+        <v>-34.01081876829222</v>
       </c>
     </row>
     <row r="10">
@@ -5406,7 +5422,7 @@
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>2008-10</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
@@ -5455,13 +5471,13 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-0.5774124374456441</v>
+        <v>-0.5757627042776047</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-0.3451933368953879</v>
+        <v>-0.3365255830162139</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.6845798786689348</v>
+        <v>0.04865772666069282</v>
       </c>
     </row>
     <row r="14">
@@ -5471,13 +5487,13 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.189176672035206</v>
+        <v>1.202436977109631</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>0.5304190741117845</v>
+        <v>0.4928100818361876</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>4.723422111329421</v>
+        <v>6.259532961263972</v>
       </c>
     </row>
     <row r="15">
@@ -5487,13 +5503,13 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>65.44715447154471</v>
+        <v>65.18218623481782</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>62.60162601626016</v>
+        <v>62.34817813765182</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>56.50406504065041</v>
+        <v>56.68016194331984</v>
       </c>
     </row>
     <row r="16">
@@ -5503,13 +5519,13 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>-7.407727877425641</v>
+        <v>-7.392292606136575</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>-8.22106512846848</v>
+        <v>-8.185644760735919</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>-7.667102791213967</v>
+        <v>-8.276024298530492</v>
       </c>
     </row>
     <row r="17">
@@ -5525,7 +5541,7 @@
         <v>-10.77835109075498</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>-12.71995100754271</v>
+        <v>-14.74439421050803</v>
       </c>
     </row>
     <row r="18">
@@ -5535,13 +5551,13 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>9.14046246715008</v>
+        <v>9.095004024940856</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>15.26612605843283</v>
+        <v>14.81756575966095</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>9.209294593663998</v>
+        <v>7.038207443820621</v>
       </c>
     </row>
     <row r="19">
@@ -5551,13 +5567,13 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>0.6555630105862931</v>
+        <v>0.6537636435369337</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>0.8666274408835086</v>
+        <v>0.8436272143092225</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.511023224712568</v>
+        <v>0.4114211549579631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Auto update: 2026-09-01
</commit_message>
<xml_diff>
--- a/docs/data.xlsx
+++ b/docs/data.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="연간 수익률&amp;금리" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="월간 수익률" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="통계" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="연간 수익률&amp;금리" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월간 수익률" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통계" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>업데이트: 2026-08-01 | Yahoo Finance Price Return</t>
+          <t>업데이트: 2026-09-01 | Yahoo Finance Price Return</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>2026</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>9.41</v>
+        <v>12.28</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>11.98</v>
+        <v>16.66</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>32.73</v>
+        <v>61.1</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>3.75</v>
@@ -1150,13 +1150,13 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>9.095000000000001</v>
+        <v>9.193</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>14.818</v>
+        <v>14.981</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>7.038</v>
+        <v>8.016</v>
       </c>
     </row>
     <row r="31">
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.824</v>
+        <v>0.831</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>1.301</v>
+        <v>1.312</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.792</v>
+        <v>0.849</v>
       </c>
     </row>
     <row r="32">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>15.127</v>
+        <v>15.102</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>18.499</v>
+        <v>18.473</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>23.108</v>
+        <v>22.335</v>
       </c>
     </row>
     <row r="33">
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>0.654</v>
+        <v>0.661</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.844</v>
+        <v>0.852</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.411</v>
+        <v>0.456</v>
       </c>
     </row>
     <row r="34">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D34" s="12" t="inlineStr">
         <is>
-          <t>2026-07 (-34.01%)</t>
+          <t>2008-10 (-23.13%)</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>월간 수익률 (2006.1 ~ 2026.07)</t>
+          <t>월간 수익률 (2006.1 ~ 2026.08)</t>
         </is>
       </c>
     </row>
@@ -5253,7 +5253,23 @@
         <v>-6.61</v>
       </c>
       <c r="D250" s="15" t="n">
-        <v>-34.01</v>
+        <v>-22.19</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="12" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B251" s="14" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="C251" s="14" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="D251" s="14" t="n">
+        <v>2.93</v>
       </c>
     </row>
   </sheetData>
@@ -5315,13 +5331,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5">
@@ -5331,13 +5347,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.8241243222789321</v>
+        <v>0.8313759452804119</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1.300548612970375</v>
+        <v>1.312172361062303</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.792271644629278</v>
+        <v>0.8485625750338993</v>
       </c>
     </row>
     <row r="6">
@@ -5347,13 +5363,13 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>1.312815216695795</v>
+        <v>1.339555553393912</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1.841223504340639</v>
+        <v>1.845703419189093</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.8323012343988134</v>
+        <v>0.8352827572794652</v>
       </c>
     </row>
     <row r="7">
@@ -5363,13 +5379,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4.366792837294682</v>
+        <v>4.359440225393032</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>5.340312017369913</v>
+        <v>5.332633280747152</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>6.670803021950943</v>
+        <v>6.447446923678635</v>
       </c>
     </row>
     <row r="8">
@@ -5379,13 +5395,13 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>15.12701412064448</v>
+        <v>15.1015439258805</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>18.49938348471067</v>
+        <v>18.47278356077355</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>23.10833952260607</v>
+        <v>22.3346113018301</v>
       </c>
     </row>
     <row r="9">
@@ -5401,7 +5417,7 @@
         <v>-16.2953145739305</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>-34.01081876829222</v>
+        <v>-23.13439957216467</v>
       </c>
     </row>
     <row r="10">
@@ -5422,7 +5438,7 @@
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2008-10</t>
         </is>
       </c>
     </row>
@@ -5471,13 +5487,13 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-0.5757627042776047</v>
+        <v>-0.5810633726544708</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-0.3365255830162139</v>
+        <v>-0.3425495837392509</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.04865772666069282</v>
+        <v>0.4844930552941536</v>
       </c>
     </row>
     <row r="14">
@@ -5487,13 +5503,13 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.202436977109631</v>
+        <v>1.217593999303062</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>0.4928100818361876</v>
+        <v>0.5019738724937164</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>6.259532961263972</v>
+        <v>4.702564139191789</v>
       </c>
     </row>
     <row r="15">
@@ -5503,13 +5519,13 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>65.18218623481782</v>
+        <v>65.32258064516128</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>62.34817813765182</v>
+        <v>62.5</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>56.68016194331984</v>
+        <v>56.85483870967742</v>
       </c>
     </row>
     <row r="16">
@@ -5519,13 +5535,13 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>-7.392292606136575</v>
+        <v>-7.376857334847509</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>-8.185644760735919</v>
+        <v>-8.150224393003358</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>-8.276024298530492</v>
+        <v>-8.234383786474245</v>
       </c>
     </row>
     <row r="17">
@@ -5541,7 +5557,7 @@
         <v>-10.77835109075498</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>-14.74439421050803</v>
+        <v>-13.83519053405983</v>
       </c>
     </row>
     <row r="18">
@@ -5551,13 +5567,13 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>9.095004024940856</v>
+        <v>9.193409172183564</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>14.81756575966095</v>
+        <v>14.98138954144166</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>7.038207443820621</v>
+        <v>8.016362764477858</v>
       </c>
     </row>
     <row r="19">
@@ -5567,13 +5583,13 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>0.6537636435369337</v>
+        <v>0.6606285683325097</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>0.8436272143092225</v>
+        <v>0.8523928340818097</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.4114211549579631</v>
+        <v>0.4559179814144521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Auto update: 2026-10-01
</commit_message>
<xml_diff>
--- a/docs/data.xlsx
+++ b/docs/data.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>업데이트: 2026-09-01 | Yahoo Finance Price Return</t>
+          <t>업데이트: 2026-10-01 | Yahoo Finance Price Return</t>
         </is>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>2026</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12.28</v>
+        <v>11.77</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>16.66</v>
+        <v>20.43</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>61.1</v>
+        <v>68.03</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>3.75</v>
@@ -1150,13 +1150,13 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>9.193</v>
+        <v>9.131</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>14.981</v>
+        <v>15.093</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>8.016</v>
+        <v>8.202</v>
       </c>
     </row>
     <row r="31">
@@ -1166,13 +1166,13 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>0.831</v>
+        <v>0.826</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>1.312</v>
+        <v>1.32</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>0.849</v>
+        <v>0.862</v>
       </c>
     </row>
     <row r="32">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>15.102</v>
+        <v>15.074</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>18.473</v>
+        <v>18.44</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>22.335</v>
+        <v>22.301</v>
       </c>
     </row>
     <row r="33">
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>0.661</v>
+        <v>0.658</v>
       </c>
       <c r="C33" s="11" t="n">
-        <v>0.852</v>
+        <v>0.859</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>0.456</v>
+        <v>0.464</v>
       </c>
     </row>
     <row r="34">
@@ -1266,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D251"/>
+  <dimension ref="A1:D252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1278,7 +1278,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>월간 수익률 (2006.1 ~ 2026.08)</t>
+          <t>월간 수익률 (2006.1 ~ 2026.09)</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,23 @@
         <v>4.18</v>
       </c>
       <c r="D251" s="14" t="n">
-        <v>2.93</v>
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="12" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B252" s="15" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="C252" s="14" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="D252" s="14" t="n">
+        <v>3.83</v>
       </c>
     </row>
   </sheetData>
@@ -5331,13 +5347,13 @@
         </is>
       </c>
       <c r="B4" s="17" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C4" s="17" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D4" s="17" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5">
@@ -5347,13 +5363,13 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>0.8313759452804119</v>
+        <v>0.8262292057347737</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>1.312172361062303</v>
+        <v>1.319875421654894</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>0.8485625750338993</v>
+        <v>0.8624143167762873</v>
       </c>
     </row>
     <row r="6">
@@ -5363,13 +5379,13 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>1.339555553393912</v>
+        <v>1.312815216695795</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>1.845703419189093</v>
+        <v>1.850183334037547</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>0.8352827572794652</v>
+        <v>0.838264280160117</v>
       </c>
     </row>
     <row r="7">
@@ -5379,13 +5395,13 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4.359440225393032</v>
+        <v>4.351400106869662</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>5.332633280747152</v>
+        <v>5.32325909285231</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>6.447446923678635</v>
+        <v>6.437882356929037</v>
       </c>
     </row>
     <row r="8">
@@ -5395,13 +5411,13 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>15.1015439258805</v>
+        <v>15.07369213831779</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>18.47278356077355</v>
+        <v>18.44031042134642</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>22.3346113018301</v>
+        <v>22.30147867070473</v>
       </c>
     </row>
     <row r="9">
@@ -5487,13 +5503,13 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>-0.5810633726544708</v>
+        <v>-0.5784419974341789</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>-0.3425495837392509</v>
+        <v>-0.3471488661197435</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.4844930552941536</v>
+        <v>0.4786889206029177</v>
       </c>
     </row>
     <row r="14">
@@ -5503,13 +5519,13 @@
         </is>
       </c>
       <c r="B14" s="20" t="n">
-        <v>1.217593999303062</v>
+        <v>1.228815693865784</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>0.5019738724937164</v>
+        <v>0.5144975300439949</v>
       </c>
       <c r="D14" s="20" t="n">
-        <v>4.702564139191789</v>
+        <v>4.71268746470144</v>
       </c>
     </row>
     <row r="15">
@@ -5519,13 +5535,13 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>65.32258064516128</v>
+        <v>65.06024096385542</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>62.5</v>
+        <v>62.65060240963856</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>56.85483870967742</v>
+        <v>57.0281124497992</v>
       </c>
     </row>
     <row r="16">
@@ -5535,13 +5551,13 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>-7.376857334847509</v>
+        <v>-7.361422063558443</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>-8.150224393003358</v>
+        <v>-8.114804025270798</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>-8.234383786474245</v>
+        <v>-8.192743274417998</v>
       </c>
     </row>
     <row r="17">
@@ -5567,13 +5583,13 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>9.193409172183564</v>
+        <v>9.131115690299341</v>
       </c>
       <c r="C18" s="20" t="n">
-        <v>14.98138954144166</v>
+        <v>15.09314617395452</v>
       </c>
       <c r="D18" s="20" t="n">
-        <v>8.016362764477858</v>
+        <v>8.202320293195209</v>
       </c>
     </row>
     <row r="19">
@@ -5583,13 +5599,13 @@
         </is>
       </c>
       <c r="B19" s="18" t="n">
-        <v>0.6606285683325097</v>
+        <v>0.6577519547194199</v>
       </c>
       <c r="C19" s="18" t="n">
-        <v>0.8523928340818097</v>
+        <v>0.858906639745291</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.4559179814144521</v>
+        <v>0.4640486827857688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>